<commit_message>
M20-8761346 Ye part add kr dia ha Library me or controller Board k BOM me
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/LCSC_Control_Board.xlsx
+++ b/Deliverables/Control_Board/BOM/LCSC_Control_Board.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="186">
   <si>
     <t>S. No.</t>
   </si>
@@ -487,13 +487,7 @@
     <t>Aliexpress</t>
   </si>
   <si>
-    <t>P=2.54mm Female Headers,SMD,ROHS</t>
-  </si>
-  <si>
     <t>J3</t>
-  </si>
-  <si>
-    <t>PHF254SMD-x</t>
   </si>
   <si>
     <t>Solder Bridge ON</t>
@@ -588,6 +582,17 @@
   </si>
   <si>
     <t xml:space="preserve">Ye part Same ha or Quantity b Zayada ha is lye merge kr dia ha isko  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">M20-8761346
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONN HEADER SMD 26POS 2.54MM
+</t>
+  </si>
+  <si>
+    <t>Harwin</t>
   </si>
 </sst>
 </file>
@@ -1509,6 +1514,84 @@
     <xf numFmtId="167" fontId="16" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1539,73 +1622,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="30" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1614,35 +1646,8 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="30" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1946,28 +1951,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="16.5" thickBot="1">
-      <c r="A1" s="110" t="s">
-        <v>173</v>
-      </c>
-      <c r="B1" s="111"/>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="111"/>
-      <c r="L1" s="111"/>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
-      <c r="O1" s="111"/>
-      <c r="P1" s="111"/>
-      <c r="Q1" s="111"/>
-      <c r="R1" s="111"/>
-      <c r="S1" s="111"/>
-      <c r="T1" s="112"/>
+      <c r="A1" s="136" t="s">
+        <v>171</v>
+      </c>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
+      <c r="F1" s="137"/>
+      <c r="G1" s="137"/>
+      <c r="H1" s="137"/>
+      <c r="I1" s="137"/>
+      <c r="J1" s="137"/>
+      <c r="K1" s="137"/>
+      <c r="L1" s="137"/>
+      <c r="M1" s="137"/>
+      <c r="N1" s="137"/>
+      <c r="O1" s="137"/>
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="R1" s="137"/>
+      <c r="S1" s="137"/>
+      <c r="T1" s="138"/>
     </row>
     <row r="2" spans="1:21" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -2007,7 +2012,7 @@
         <v>11</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="N2" s="12" t="s">
         <v>12</v>
@@ -2016,10 +2021,10 @@
         <v>13</v>
       </c>
       <c r="P2" s="20" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="Q2" s="20" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>14</v>
@@ -2035,7 +2040,7 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="115" t="s">
+      <c r="B3" s="141" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="32" t="s">
@@ -2096,12 +2101,12 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="116"/>
+      <c r="B4" s="142"/>
       <c r="C4" s="41" t="s">
         <v>27</v>
       </c>
       <c r="D4" s="94" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E4" s="25" t="s">
         <v>28</v>
@@ -2155,7 +2160,7 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="116"/>
+      <c r="B5" s="142"/>
       <c r="C5" s="41" t="s">
         <v>33</v>
       </c>
@@ -2215,7 +2220,7 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="116"/>
+      <c r="B6" s="142"/>
       <c r="C6" s="41" t="s">
         <v>39</v>
       </c>
@@ -2275,7 +2280,7 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="117"/>
+      <c r="B7" s="143"/>
       <c r="C7" s="51" t="s">
         <v>46</v>
       </c>
@@ -2397,7 +2402,7 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="115" t="s">
+      <c r="B9" s="141" t="s">
         <v>61</v>
       </c>
       <c r="C9" s="32" t="s">
@@ -2459,7 +2464,7 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="117"/>
+      <c r="B10" s="143"/>
       <c r="C10" s="51" t="s">
         <v>68</v>
       </c>
@@ -2519,7 +2524,7 @@
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="115" t="s">
+      <c r="B11" s="141" t="s">
         <v>74</v>
       </c>
       <c r="C11" s="32" t="s">
@@ -2581,7 +2586,7 @@
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="116"/>
+      <c r="B12" s="142"/>
       <c r="C12" s="41" t="s">
         <v>81</v>
       </c>
@@ -2641,7 +2646,7 @@
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="116"/>
+      <c r="B13" s="142"/>
       <c r="C13" s="41" t="s">
         <v>86</v>
       </c>
@@ -2701,7 +2706,7 @@
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="116"/>
+      <c r="B14" s="142"/>
       <c r="C14" s="41" t="s">
         <v>91</v>
       </c>
@@ -2761,7 +2766,7 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="118"/>
+      <c r="B15" s="144"/>
       <c r="C15" s="96" t="s">
         <v>96</v>
       </c>
@@ -2821,7 +2826,7 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="118"/>
+      <c r="B16" s="144"/>
       <c r="C16" s="96" t="s">
         <v>101</v>
       </c>
@@ -2881,7 +2886,7 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="117"/>
+      <c r="B17" s="143"/>
       <c r="C17" s="51" t="s">
         <v>106</v>
       </c>
@@ -3003,7 +3008,7 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="115" t="s">
+      <c r="B19" s="141" t="s">
         <v>118</v>
       </c>
       <c r="C19" s="101" t="s">
@@ -3013,21 +3018,21 @@
         <v>120</v>
       </c>
       <c r="E19" s="103" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F19" s="102" t="s">
         <v>121</v>
       </c>
       <c r="G19" s="105" t="s">
-        <v>175</v>
-      </c>
-      <c r="H19" s="122" t="s">
-        <v>170</v>
-      </c>
-      <c r="I19" s="122" t="s">
-        <v>176</v>
-      </c>
-      <c r="J19" s="122" t="s">
+        <v>173</v>
+      </c>
+      <c r="H19" s="110" t="s">
+        <v>168</v>
+      </c>
+      <c r="I19" s="110" t="s">
+        <v>174</v>
+      </c>
+      <c r="J19" s="110" t="s">
         <v>60</v>
       </c>
       <c r="K19" s="105">
@@ -3040,20 +3045,20 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N19" s="123" t="s">
+      <c r="N19" s="111" t="s">
         <v>145</v>
       </c>
-      <c r="O19" s="124">
+      <c r="O19" s="112">
         <v>21.26</v>
       </c>
       <c r="P19" s="106">
         <f t="shared" si="1"/>
         <v>21.26</v>
       </c>
-      <c r="Q19" s="124">
+      <c r="Q19" s="112">
         <v>21.26</v>
       </c>
-      <c r="R19" s="125">
+      <c r="R19" s="113">
         <f t="shared" si="2"/>
         <v>106.30000000000001</v>
       </c>
@@ -3065,7 +3070,7 @@
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="116"/>
+      <c r="B20" s="142"/>
       <c r="C20" s="83" t="s">
         <v>122</v>
       </c>
@@ -3125,60 +3130,60 @@
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="116"/>
-      <c r="C21" s="152" t="s">
+      <c r="B21" s="142"/>
+      <c r="C21" s="132" t="s">
         <v>128</v>
       </c>
-      <c r="D21" s="126" t="s">
+      <c r="D21" s="114" t="s">
         <v>129</v>
       </c>
-      <c r="E21" s="126" t="s">
+      <c r="E21" s="114" t="s">
         <v>124</v>
       </c>
-      <c r="F21" s="126" t="s">
+      <c r="F21" s="114" t="s">
         <v>130</v>
       </c>
-      <c r="G21" s="127" t="s">
+      <c r="G21" s="115" t="s">
         <v>131</v>
       </c>
-      <c r="H21" s="127" t="s">
+      <c r="H21" s="115" t="s">
         <v>24</v>
       </c>
-      <c r="I21" s="126" t="s">
+      <c r="I21" s="114" t="s">
         <v>24</v>
       </c>
-      <c r="J21" s="127" t="s">
+      <c r="J21" s="115" t="s">
         <v>60</v>
       </c>
-      <c r="K21" s="128">
+      <c r="K21" s="116">
         <v>10</v>
       </c>
-      <c r="L21" s="129">
+      <c r="L21" s="117">
         <v>1</v>
       </c>
-      <c r="M21" s="129">
+      <c r="M21" s="117">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N21" s="130" t="s">
+      <c r="N21" s="118" t="s">
         <v>150</v>
       </c>
-      <c r="O21" s="131">
+      <c r="O21" s="119">
         <v>17.38</v>
       </c>
-      <c r="P21" s="132">
+      <c r="P21" s="120">
         <f t="shared" si="1"/>
         <v>17.38</v>
       </c>
-      <c r="Q21" s="132">
+      <c r="Q21" s="120">
         <v>1.738</v>
       </c>
-      <c r="R21" s="133">
+      <c r="R21" s="121">
         <f t="shared" si="2"/>
         <v>17.38</v>
       </c>
       <c r="S21" s="22" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="T21" s="48"/>
       <c r="U21" s="17"/>
@@ -3187,60 +3192,60 @@
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="117"/>
-      <c r="C22" s="153" t="s">
+      <c r="B22" s="143"/>
+      <c r="C22" s="133" t="s">
         <v>132</v>
       </c>
-      <c r="D22" s="134" t="s">
+      <c r="D22" s="122" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="134" t="s">
+      <c r="E22" s="122" t="s">
         <v>134</v>
       </c>
-      <c r="F22" s="134" t="s">
+      <c r="F22" s="122" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="134" t="s">
+      <c r="G22" s="122" t="s">
         <v>136</v>
       </c>
-      <c r="H22" s="134" t="s">
+      <c r="H22" s="122" t="s">
         <v>137</v>
       </c>
-      <c r="I22" s="134" t="s">
+      <c r="I22" s="122" t="s">
         <v>24</v>
       </c>
-      <c r="J22" s="135" t="s">
+      <c r="J22" s="123" t="s">
         <v>60</v>
       </c>
-      <c r="K22" s="136">
+      <c r="K22" s="124">
         <v>10</v>
       </c>
-      <c r="L22" s="137">
+      <c r="L22" s="125">
         <v>1</v>
       </c>
-      <c r="M22" s="137">
+      <c r="M22" s="125">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N22" s="138" t="s">
+      <c r="N22" s="126" t="s">
         <v>150</v>
       </c>
-      <c r="O22" s="139">
+      <c r="O22" s="127">
         <v>9.4499999999999993</v>
       </c>
-      <c r="P22" s="139">
+      <c r="P22" s="127">
         <f t="shared" si="1"/>
         <v>9.4499999999999993</v>
       </c>
-      <c r="Q22" s="139">
+      <c r="Q22" s="127">
         <v>0.94499999999999995</v>
       </c>
-      <c r="R22" s="140">
+      <c r="R22" s="128">
         <f t="shared" si="2"/>
         <v>9.4499999999999993</v>
       </c>
       <c r="S22" s="30" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="T22" s="61"/>
       <c r="U22" s="17"/>
@@ -3249,7 +3254,7 @@
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="115" t="s">
+      <c r="B23" s="141" t="s">
         <v>138</v>
       </c>
       <c r="C23" s="101" t="s">
@@ -3265,7 +3270,7 @@
         <v>141</v>
       </c>
       <c r="G23" s="103" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H23" s="104"/>
       <c r="I23" s="105"/>
@@ -3291,7 +3296,7 @@
       </c>
       <c r="S23" s="107"/>
       <c r="T23" s="108" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="U23" s="17"/>
     </row>
@@ -3299,55 +3304,55 @@
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="117"/>
-      <c r="C24" s="153" t="s">
+      <c r="B24" s="143"/>
+      <c r="C24" s="133" t="s">
         <v>142</v>
       </c>
-      <c r="D24" s="134" t="s">
+      <c r="D24" s="122" t="s">
         <v>143</v>
       </c>
-      <c r="E24" s="134" t="s">
+      <c r="E24" s="122" t="s">
         <v>115</v>
       </c>
-      <c r="F24" s="134" t="s">
+      <c r="F24" s="122" t="s">
         <v>144</v>
       </c>
-      <c r="G24" s="134" t="s">
-        <v>170</v>
-      </c>
-      <c r="H24" s="134" t="s">
+      <c r="G24" s="122" t="s">
+        <v>168</v>
+      </c>
+      <c r="H24" s="122" t="s">
         <v>24</v>
       </c>
-      <c r="I24" s="134" t="s">
-        <v>170</v>
-      </c>
-      <c r="J24" s="134" t="s">
-        <v>171</v>
-      </c>
-      <c r="K24" s="136">
+      <c r="I24" s="122" t="s">
+        <v>168</v>
+      </c>
+      <c r="J24" s="122" t="s">
+        <v>169</v>
+      </c>
+      <c r="K24" s="124">
         <v>7</v>
       </c>
-      <c r="L24" s="137">
+      <c r="L24" s="125">
         <v>1</v>
       </c>
-      <c r="M24" s="137">
+      <c r="M24" s="125">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N24" s="138" t="s">
+      <c r="N24" s="126" t="s">
         <v>145</v>
       </c>
-      <c r="O24" s="141">
+      <c r="O24" s="129">
         <v>0.86619999999999997</v>
       </c>
-      <c r="P24" s="139">
+      <c r="P24" s="127">
         <f t="shared" si="1"/>
         <v>0.86619999999999997</v>
       </c>
-      <c r="Q24" s="141">
+      <c r="Q24" s="129">
         <v>0.86619999999999997</v>
       </c>
-      <c r="R24" s="140">
+      <c r="R24" s="128">
         <f t="shared" si="2"/>
         <v>6.0633999999999997</v>
       </c>
@@ -3359,61 +3364,61 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="119" t="s">
+      <c r="B25" s="145" t="s">
         <v>146</v>
       </c>
       <c r="C25" s="154" t="s">
+        <v>175</v>
+      </c>
+      <c r="D25" s="130" t="s">
         <v>177</v>
       </c>
-      <c r="D25" s="142" t="s">
-        <v>179</v>
-      </c>
-      <c r="E25" s="142" t="s">
+      <c r="E25" s="130" t="s">
         <v>147</v>
       </c>
-      <c r="F25" s="142" t="s">
+      <c r="F25" s="130" t="s">
         <v>148</v>
       </c>
-      <c r="G25" s="142" t="s">
+      <c r="G25" s="130" t="s">
         <v>149</v>
       </c>
-      <c r="H25" s="142" t="s">
-        <v>170</v>
-      </c>
-      <c r="I25" s="142" t="s">
+      <c r="H25" s="130" t="s">
+        <v>168</v>
+      </c>
+      <c r="I25" s="130" t="s">
         <v>24</v>
       </c>
-      <c r="J25" s="142" t="s">
-        <v>171</v>
-      </c>
-      <c r="K25" s="143">
+      <c r="J25" s="130" t="s">
+        <v>169</v>
+      </c>
+      <c r="K25" s="152">
         <v>5</v>
       </c>
-      <c r="L25" s="144">
+      <c r="L25" s="131">
         <v>2</v>
       </c>
-      <c r="M25" s="144">
+      <c r="M25" s="131">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N25" s="145" t="s">
+      <c r="N25" s="146" t="s">
         <v>150</v>
       </c>
-      <c r="O25" s="146">
+      <c r="O25" s="148">
         <v>11.53</v>
       </c>
-      <c r="P25" s="146">
+      <c r="P25" s="148">
         <v>11.53</v>
       </c>
-      <c r="Q25" s="146">
+      <c r="Q25" s="148">
         <v>2.306</v>
       </c>
-      <c r="R25" s="147">
+      <c r="R25" s="150">
         <f t="shared" si="2"/>
         <v>11.530000000000001</v>
       </c>
-      <c r="S25" s="121" t="s">
-        <v>184</v>
+      <c r="S25" s="134" t="s">
+        <v>182</v>
       </c>
       <c r="T25" s="100"/>
       <c r="U25" s="17"/>
@@ -3422,45 +3427,45 @@
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="119"/>
-      <c r="C26" s="152" t="s">
+      <c r="B26" s="145"/>
+      <c r="C26" s="132" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="130" t="s">
+        <v>179</v>
+      </c>
+      <c r="E26" s="114" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="142" t="s">
-        <v>181</v>
-      </c>
-      <c r="E26" s="126" t="s">
+      <c r="F26" s="114" t="s">
         <v>180</v>
       </c>
-      <c r="F26" s="126" t="s">
-        <v>182</v>
-      </c>
-      <c r="G26" s="126" t="s">
+      <c r="G26" s="114" t="s">
         <v>149</v>
       </c>
-      <c r="H26" s="142" t="s">
-        <v>170</v>
-      </c>
-      <c r="I26" s="142" t="s">
-        <v>176</v>
-      </c>
-      <c r="J26" s="142" t="s">
-        <v>171</v>
-      </c>
-      <c r="K26" s="148"/>
-      <c r="L26" s="144">
+      <c r="H26" s="130" t="s">
+        <v>168</v>
+      </c>
+      <c r="I26" s="130" t="s">
+        <v>174</v>
+      </c>
+      <c r="J26" s="130" t="s">
+        <v>169</v>
+      </c>
+      <c r="K26" s="153"/>
+      <c r="L26" s="131">
         <v>1</v>
       </c>
-      <c r="M26" s="144">
+      <c r="M26" s="131">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N26" s="149"/>
-      <c r="O26" s="150"/>
-      <c r="P26" s="150"/>
-      <c r="Q26" s="150"/>
+      <c r="N26" s="147"/>
+      <c r="O26" s="149"/>
+      <c r="P26" s="149"/>
+      <c r="Q26" s="149"/>
       <c r="R26" s="151"/>
-      <c r="S26" s="120"/>
+      <c r="S26" s="135"/>
       <c r="T26" s="100"/>
       <c r="U26" s="17"/>
     </row>
@@ -3468,57 +3473,49 @@
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="116"/>
-      <c r="C27" s="152" t="s">
+      <c r="B27" s="142"/>
+      <c r="C27" s="132" t="s">
+        <v>184</v>
+      </c>
+      <c r="D27" s="114" t="s">
         <v>151</v>
       </c>
-      <c r="D27" s="126" t="s">
-        <v>152</v>
-      </c>
-      <c r="E27" s="126" t="s">
-        <v>153</v>
-      </c>
-      <c r="F27" s="126" t="s">
-        <v>153</v>
-      </c>
-      <c r="G27" s="126" t="s">
-        <v>149</v>
-      </c>
-      <c r="H27" s="126" t="s">
-        <v>172</v>
-      </c>
-      <c r="I27" s="126" t="s">
+      <c r="E27" s="114" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="114" t="s">
+        <v>183</v>
+      </c>
+      <c r="G27" s="114" t="s">
+        <v>185</v>
+      </c>
+      <c r="H27" s="114" t="s">
+        <v>170</v>
+      </c>
+      <c r="I27" s="114" t="s">
+        <v>167</v>
+      </c>
+      <c r="J27" s="114" t="s">
         <v>169</v>
       </c>
-      <c r="J27" s="126" t="s">
-        <v>171</v>
-      </c>
-      <c r="K27" s="129">
-        <v>5</v>
-      </c>
-      <c r="L27" s="129">
+      <c r="K27" s="117"/>
+      <c r="L27" s="117">
         <v>1</v>
       </c>
-      <c r="M27" s="129">
+      <c r="M27" s="117">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N27" s="130" t="s">
-        <v>150</v>
-      </c>
-      <c r="O27" s="132">
-        <v>36.9</v>
-      </c>
-      <c r="P27" s="132">
+      <c r="N27" s="118"/>
+      <c r="O27" s="120"/>
+      <c r="P27" s="120">
         <f t="shared" si="1"/>
-        <v>36.9</v>
-      </c>
-      <c r="Q27" s="132">
-        <v>7.38</v>
-      </c>
-      <c r="R27" s="133">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="120"/>
+      <c r="R27" s="121">
         <f t="shared" si="2"/>
-        <v>36.9</v>
+        <v>0</v>
       </c>
       <c r="S27" s="78"/>
       <c r="T27" s="48"/>
@@ -3528,33 +3525,33 @@
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="116"/>
+      <c r="B28" s="142"/>
       <c r="C28" s="84" t="s">
+        <v>152</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E28" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="D28" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="E28" s="23" t="s">
-        <v>156</v>
-      </c>
       <c r="F28" s="85" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J28" s="23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="L28" s="86">
         <v>5</v>
@@ -3564,22 +3561,22 @@
         <v>25</v>
       </c>
       <c r="N28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="P28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="Q28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="R28" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S28" s="87" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="T28" s="88"/>
       <c r="U28" s="17"/>
@@ -3588,33 +3585,33 @@
       <c r="A29" s="6">
         <v>27</v>
       </c>
-      <c r="B29" s="117"/>
+      <c r="B29" s="143"/>
       <c r="C29" s="89" t="s">
+        <v>156</v>
+      </c>
+      <c r="D29" s="90" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" s="31" t="s">
         <v>158</v>
       </c>
-      <c r="D29" s="90" t="s">
-        <v>159</v>
-      </c>
-      <c r="E29" s="31" t="s">
-        <v>160</v>
-      </c>
       <c r="F29" s="90" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J29" s="31" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="L29" s="91">
         <v>3</v>
@@ -3624,22 +3621,22 @@
         <v>15</v>
       </c>
       <c r="N29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="P29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="Q29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="R29" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S29" s="92" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="T29" s="93"/>
       <c r="U29" s="17"/>
@@ -3654,19 +3651,19 @@
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
-      <c r="L30" s="113" t="s">
-        <v>161</v>
-      </c>
-      <c r="M30" s="113"/>
-      <c r="N30" s="113"/>
-      <c r="O30" s="113"/>
+      <c r="L30" s="139" t="s">
+        <v>159</v>
+      </c>
+      <c r="M30" s="139"/>
+      <c r="N30" s="139"/>
+      <c r="O30" s="139"/>
       <c r="P30" s="99">
         <f>SUM(P3:P27)</f>
-        <v>98.856999999999999</v>
+        <v>61.957000000000001</v>
       </c>
       <c r="R30" s="15">
         <f>SUM(R3:R27)</f>
-        <v>200.8844</v>
+        <v>163.98439999999999</v>
       </c>
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
@@ -3682,15 +3679,15 @@
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
-      <c r="L31" s="114" t="s">
-        <v>162</v>
-      </c>
-      <c r="M31" s="114"/>
-      <c r="N31" s="114"/>
-      <c r="O31" s="114"/>
+      <c r="L31" s="140" t="s">
+        <v>160</v>
+      </c>
+      <c r="M31" s="140"/>
+      <c r="N31" s="140"/>
+      <c r="O31" s="140"/>
       <c r="R31" s="16">
         <f>R30/5</f>
-        <v>40.176879999999997</v>
+        <v>32.796880000000002</v>
       </c>
       <c r="S31" s="7"/>
       <c r="T31" s="7"/>
@@ -3991,13 +3988,12 @@
     <hyperlink ref="N7" r:id="rId15"/>
     <hyperlink ref="N21" r:id="rId16"/>
     <hyperlink ref="N25" r:id="rId17"/>
-    <hyperlink ref="N27" r:id="rId18"/>
-    <hyperlink ref="N22" r:id="rId19"/>
-    <hyperlink ref="N15" r:id="rId20"/>
-    <hyperlink ref="N16" r:id="rId21"/>
+    <hyperlink ref="N22" r:id="rId18"/>
+    <hyperlink ref="N15" r:id="rId19"/>
+    <hyperlink ref="N16" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId21"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Controller Board k BOM me Male header ka link add kr dia ha Female header ki jaga
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/LCSC_Control_Board.xlsx
+++ b/Deliverables/Control_Board/BOM/LCSC_Control_Board.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="186">
   <si>
     <t>S. No.</t>
   </si>
@@ -584,15 +584,15 @@
     <t xml:space="preserve">Ye part Same ha or Quantity b Zayada ha is lye merge kr dia ha isko  </t>
   </si>
   <si>
-    <t xml:space="preserve">M20-8761346
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">CONN HEADER SMD 26POS 2.54MM
 </t>
   </si>
   <si>
-    <t>Harwin</t>
+    <t xml:space="preserve">95278-101A26LF
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amphenol </t>
   </si>
 </sst>
 </file>
@@ -786,7 +786,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -1182,6 +1182,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1191,7 +1200,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1577,15 +1586,18 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1601,9 +1613,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1646,8 +1655,11 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1951,28 +1963,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="16.5" thickBot="1">
-      <c r="A1" s="136" t="s">
+      <c r="A1" s="137" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="137"/>
-      <c r="C1" s="137"/>
-      <c r="D1" s="137"/>
-      <c r="E1" s="137"/>
-      <c r="F1" s="137"/>
-      <c r="G1" s="137"/>
-      <c r="H1" s="137"/>
-      <c r="I1" s="137"/>
-      <c r="J1" s="137"/>
-      <c r="K1" s="137"/>
-      <c r="L1" s="137"/>
-      <c r="M1" s="137"/>
-      <c r="N1" s="137"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="137"/>
-      <c r="Q1" s="137"/>
-      <c r="R1" s="137"/>
-      <c r="S1" s="137"/>
-      <c r="T1" s="138"/>
+      <c r="B1" s="138"/>
+      <c r="C1" s="138"/>
+      <c r="D1" s="138"/>
+      <c r="E1" s="138"/>
+      <c r="F1" s="138"/>
+      <c r="G1" s="138"/>
+      <c r="H1" s="138"/>
+      <c r="I1" s="138"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="138"/>
+      <c r="L1" s="138"/>
+      <c r="M1" s="138"/>
+      <c r="N1" s="138"/>
+      <c r="O1" s="138"/>
+      <c r="P1" s="138"/>
+      <c r="Q1" s="138"/>
+      <c r="R1" s="138"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="139"/>
     </row>
     <row r="2" spans="1:21" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -3131,7 +3143,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="142"/>
-      <c r="C21" s="132" t="s">
+      <c r="C21" s="131" t="s">
         <v>128</v>
       </c>
       <c r="D21" s="114" t="s">
@@ -3193,7 +3205,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="143"/>
-      <c r="C22" s="133" t="s">
+      <c r="C22" s="132" t="s">
         <v>132</v>
       </c>
       <c r="D22" s="122" t="s">
@@ -3305,7 +3317,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="143"/>
-      <c r="C24" s="133" t="s">
+      <c r="C24" s="132" t="s">
         <v>142</v>
       </c>
       <c r="D24" s="122" t="s">
@@ -3367,7 +3379,7 @@
       <c r="B25" s="145" t="s">
         <v>146</v>
       </c>
-      <c r="C25" s="154" t="s">
+      <c r="C25" s="134" t="s">
         <v>175</v>
       </c>
       <c r="D25" s="130" t="s">
@@ -3394,10 +3406,10 @@
       <c r="K25" s="152">
         <v>5</v>
       </c>
-      <c r="L25" s="131">
+      <c r="L25" s="133">
         <v>2</v>
       </c>
-      <c r="M25" s="131">
+      <c r="M25" s="133">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -3417,7 +3429,7 @@
         <f t="shared" si="2"/>
         <v>11.530000000000001</v>
       </c>
-      <c r="S25" s="134" t="s">
+      <c r="S25" s="135" t="s">
         <v>182</v>
       </c>
       <c r="T25" s="100"/>
@@ -3428,7 +3440,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="145"/>
-      <c r="C26" s="132" t="s">
+      <c r="C26" s="131" t="s">
         <v>176</v>
       </c>
       <c r="D26" s="130" t="s">
@@ -3453,10 +3465,10 @@
         <v>169</v>
       </c>
       <c r="K26" s="153"/>
-      <c r="L26" s="131">
+      <c r="L26" s="133">
         <v>1</v>
       </c>
-      <c r="M26" s="131">
+      <c r="M26" s="133">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -3465,7 +3477,7 @@
       <c r="P26" s="149"/>
       <c r="Q26" s="149"/>
       <c r="R26" s="151"/>
-      <c r="S26" s="135"/>
+      <c r="S26" s="136"/>
       <c r="T26" s="100"/>
       <c r="U26" s="17"/>
     </row>
@@ -3474,8 +3486,8 @@
         <v>25</v>
       </c>
       <c r="B27" s="142"/>
-      <c r="C27" s="132" t="s">
-        <v>184</v>
+      <c r="C27" s="131" t="s">
+        <v>183</v>
       </c>
       <c r="D27" s="114" t="s">
         <v>151</v>
@@ -3484,7 +3496,7 @@
         <v>115</v>
       </c>
       <c r="F27" s="114" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G27" s="114" t="s">
         <v>185</v>
@@ -3498,7 +3510,9 @@
       <c r="J27" s="114" t="s">
         <v>169</v>
       </c>
-      <c r="K27" s="117"/>
+      <c r="K27" s="117">
+        <v>10</v>
+      </c>
       <c r="L27" s="117">
         <v>1</v>
       </c>
@@ -3506,16 +3520,22 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N27" s="118"/>
-      <c r="O27" s="120"/>
+      <c r="N27" s="126" t="s">
+        <v>150</v>
+      </c>
+      <c r="O27" s="120">
+        <v>5.04</v>
+      </c>
       <c r="P27" s="120">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q27" s="120"/>
+        <v>5.04</v>
+      </c>
+      <c r="Q27" s="120">
+        <v>0.504</v>
+      </c>
       <c r="R27" s="121">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.04</v>
       </c>
       <c r="S27" s="78"/>
       <c r="T27" s="48"/>
@@ -3582,7 +3602,7 @@
       <c r="U28" s="17"/>
     </row>
     <row r="29" spans="1:21" ht="15.75" thickBot="1">
-      <c r="A29" s="6">
+      <c r="A29" s="155">
         <v>27</v>
       </c>
       <c r="B29" s="143"/>
@@ -3651,19 +3671,19 @@
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
-      <c r="L30" s="139" t="s">
+      <c r="L30" s="154" t="s">
         <v>159</v>
       </c>
-      <c r="M30" s="139"/>
-      <c r="N30" s="139"/>
-      <c r="O30" s="139"/>
+      <c r="M30" s="154"/>
+      <c r="N30" s="154"/>
+      <c r="O30" s="154"/>
       <c r="P30" s="99">
         <f>SUM(P3:P27)</f>
-        <v>61.957000000000001</v>
+        <v>66.997</v>
       </c>
       <c r="R30" s="15">
         <f>SUM(R3:R27)</f>
-        <v>163.98439999999999</v>
+        <v>169.02439999999999</v>
       </c>
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
@@ -3687,7 +3707,7 @@
       <c r="O31" s="140"/>
       <c r="R31" s="16">
         <f>R30/5</f>
-        <v>32.796880000000002</v>
+        <v>33.804879999999997</v>
       </c>
       <c r="S31" s="7"/>
       <c r="T31" s="7"/>
@@ -3991,9 +4011,10 @@
     <hyperlink ref="N22" r:id="rId18"/>
     <hyperlink ref="N15" r:id="rId19"/>
     <hyperlink ref="N16" r:id="rId20"/>
+    <hyperlink ref="N27" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId21"/>
+  <pageSetup orientation="portrait" r:id="rId22"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
#8 Custom supplier ki price update kr di BOM me kuch parts out of stock han quotation me
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/LCSC_Control_Board.xlsx
+++ b/Deliverables/Control_Board/BOM/LCSC_Control_Board.xlsx
@@ -1598,6 +1598,9 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1613,6 +1616,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1653,12 +1659,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1963,28 +1963,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="16.5" thickBot="1">
-      <c r="A1" s="137" t="s">
+      <c r="A1" s="138" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
-      <c r="N1" s="138"/>
-      <c r="O1" s="138"/>
-      <c r="P1" s="138"/>
-      <c r="Q1" s="138"/>
-      <c r="R1" s="138"/>
-      <c r="S1" s="138"/>
-      <c r="T1" s="139"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="139"/>
+      <c r="M1" s="139"/>
+      <c r="N1" s="139"/>
+      <c r="O1" s="139"/>
+      <c r="P1" s="139"/>
+      <c r="Q1" s="139"/>
+      <c r="R1" s="139"/>
+      <c r="S1" s="139"/>
+      <c r="T1" s="140"/>
     </row>
     <row r="2" spans="1:21" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -2052,7 +2052,7 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="141" t="s">
+      <c r="B3" s="143" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="32" t="s">
@@ -2113,7 +2113,7 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="142"/>
+      <c r="B4" s="144"/>
       <c r="C4" s="41" t="s">
         <v>27</v>
       </c>
@@ -2172,7 +2172,7 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="142"/>
+      <c r="B5" s="144"/>
       <c r="C5" s="41" t="s">
         <v>33</v>
       </c>
@@ -2232,7 +2232,7 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="142"/>
+      <c r="B6" s="144"/>
       <c r="C6" s="41" t="s">
         <v>39</v>
       </c>
@@ -2292,7 +2292,7 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="143"/>
+      <c r="B7" s="145"/>
       <c r="C7" s="51" t="s">
         <v>46</v>
       </c>
@@ -2414,7 +2414,7 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="141" t="s">
+      <c r="B9" s="143" t="s">
         <v>61</v>
       </c>
       <c r="C9" s="32" t="s">
@@ -2476,7 +2476,7 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="143"/>
+      <c r="B10" s="145"/>
       <c r="C10" s="51" t="s">
         <v>68</v>
       </c>
@@ -2536,7 +2536,7 @@
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="141" t="s">
+      <c r="B11" s="143" t="s">
         <v>74</v>
       </c>
       <c r="C11" s="32" t="s">
@@ -2598,7 +2598,7 @@
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="142"/>
+      <c r="B12" s="144"/>
       <c r="C12" s="41" t="s">
         <v>81</v>
       </c>
@@ -2658,7 +2658,7 @@
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="142"/>
+      <c r="B13" s="144"/>
       <c r="C13" s="41" t="s">
         <v>86</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="142"/>
+      <c r="B14" s="144"/>
       <c r="C14" s="41" t="s">
         <v>91</v>
       </c>
@@ -2778,7 +2778,7 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="144"/>
+      <c r="B15" s="146"/>
       <c r="C15" s="96" t="s">
         <v>96</v>
       </c>
@@ -2838,7 +2838,7 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="144"/>
+      <c r="B16" s="146"/>
       <c r="C16" s="96" t="s">
         <v>101</v>
       </c>
@@ -2898,7 +2898,7 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="143"/>
+      <c r="B17" s="145"/>
       <c r="C17" s="51" t="s">
         <v>106</v>
       </c>
@@ -3020,7 +3020,7 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="141" t="s">
+      <c r="B19" s="143" t="s">
         <v>118</v>
       </c>
       <c r="C19" s="101" t="s">
@@ -3082,7 +3082,7 @@
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="142"/>
+      <c r="B20" s="144"/>
       <c r="C20" s="83" t="s">
         <v>122</v>
       </c>
@@ -3142,7 +3142,7 @@
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="142"/>
+      <c r="B21" s="144"/>
       <c r="C21" s="131" t="s">
         <v>128</v>
       </c>
@@ -3197,14 +3197,16 @@
       <c r="S21" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="T21" s="48"/>
+      <c r="T21" s="48">
+        <v>1.1904999999999999</v>
+      </c>
       <c r="U21" s="17"/>
     </row>
     <row r="22" spans="1:21" ht="15.75" thickBot="1">
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="143"/>
+      <c r="B22" s="145"/>
       <c r="C22" s="132" t="s">
         <v>132</v>
       </c>
@@ -3259,14 +3261,16 @@
       <c r="S22" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="T22" s="61"/>
+      <c r="T22" s="61">
+        <v>0.79400000000000004</v>
+      </c>
       <c r="U22" s="17"/>
     </row>
     <row r="23" spans="1:21" ht="15.75" thickBot="1">
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="141" t="s">
+      <c r="B23" s="143" t="s">
         <v>138</v>
       </c>
       <c r="C23" s="101" t="s">
@@ -3316,7 +3320,7 @@
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="143"/>
+      <c r="B24" s="145"/>
       <c r="C24" s="132" t="s">
         <v>142</v>
       </c>
@@ -3376,7 +3380,7 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="145" t="s">
+      <c r="B25" s="147" t="s">
         <v>146</v>
       </c>
       <c r="C25" s="134" t="s">
@@ -3403,7 +3407,7 @@
       <c r="J25" s="130" t="s">
         <v>169</v>
       </c>
-      <c r="K25" s="152">
+      <c r="K25" s="154">
         <v>5</v>
       </c>
       <c r="L25" s="133">
@@ -3413,23 +3417,23 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="N25" s="146" t="s">
+      <c r="N25" s="148" t="s">
         <v>150</v>
       </c>
-      <c r="O25" s="148">
+      <c r="O25" s="150">
         <v>11.53</v>
       </c>
-      <c r="P25" s="148">
+      <c r="P25" s="150">
         <v>11.53</v>
       </c>
-      <c r="Q25" s="148">
+      <c r="Q25" s="150">
         <v>2.306</v>
       </c>
-      <c r="R25" s="150">
+      <c r="R25" s="152">
         <f t="shared" si="2"/>
         <v>11.530000000000001</v>
       </c>
-      <c r="S25" s="135" t="s">
+      <c r="S25" s="136" t="s">
         <v>182</v>
       </c>
       <c r="T25" s="100"/>
@@ -3439,7 +3443,7 @@
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="145"/>
+      <c r="B26" s="147"/>
       <c r="C26" s="131" t="s">
         <v>176</v>
       </c>
@@ -3464,7 +3468,7 @@
       <c r="J26" s="130" t="s">
         <v>169</v>
       </c>
-      <c r="K26" s="153"/>
+      <c r="K26" s="155"/>
       <c r="L26" s="133">
         <v>1</v>
       </c>
@@ -3472,12 +3476,12 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N26" s="147"/>
-      <c r="O26" s="149"/>
-      <c r="P26" s="149"/>
-      <c r="Q26" s="149"/>
-      <c r="R26" s="151"/>
-      <c r="S26" s="136"/>
+      <c r="N26" s="149"/>
+      <c r="O26" s="151"/>
+      <c r="P26" s="151"/>
+      <c r="Q26" s="151"/>
+      <c r="R26" s="153"/>
+      <c r="S26" s="137"/>
       <c r="T26" s="100"/>
       <c r="U26" s="17"/>
     </row>
@@ -3485,7 +3489,7 @@
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="142"/>
+      <c r="B27" s="144"/>
       <c r="C27" s="131" t="s">
         <v>183</v>
       </c>
@@ -3545,7 +3549,7 @@
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="142"/>
+      <c r="B28" s="144"/>
       <c r="C28" s="84" t="s">
         <v>152</v>
       </c>
@@ -3602,10 +3606,10 @@
       <c r="U28" s="17"/>
     </row>
     <row r="29" spans="1:21" ht="15.75" thickBot="1">
-      <c r="A29" s="155">
+      <c r="A29" s="135">
         <v>27</v>
       </c>
-      <c r="B29" s="143"/>
+      <c r="B29" s="145"/>
       <c r="C29" s="89" t="s">
         <v>156</v>
       </c>
@@ -3671,12 +3675,12 @@
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
-      <c r="L30" s="154" t="s">
+      <c r="L30" s="141" t="s">
         <v>159</v>
       </c>
-      <c r="M30" s="154"/>
-      <c r="N30" s="154"/>
-      <c r="O30" s="154"/>
+      <c r="M30" s="141"/>
+      <c r="N30" s="141"/>
+      <c r="O30" s="141"/>
       <c r="P30" s="99">
         <f>SUM(P3:P27)</f>
         <v>66.997</v>
@@ -3699,12 +3703,12 @@
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
-      <c r="L31" s="140" t="s">
+      <c r="L31" s="142" t="s">
         <v>160</v>
       </c>
-      <c r="M31" s="140"/>
-      <c r="N31" s="140"/>
-      <c r="O31" s="140"/>
+      <c r="M31" s="142"/>
+      <c r="N31" s="142"/>
+      <c r="O31" s="142"/>
       <c r="R31" s="16">
         <f>R30/5</f>
         <v>33.804879999999997</v>

</xml_diff>